<commit_message>
chore: 체크리스트 9/7 R33·R36 완료 처리 (34→36)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3rd_host_ai_체크리스트.xlsx
+++ b/3rd_host_ai_체크리스트.xlsx
@@ -2434,9 +2434,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3753,7 +3753,7 @@
       </c>
       <c r="E33" s="124" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F33" s="130" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="E36" s="124" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F36" s="130" t="inlineStr">
@@ -17426,7 +17426,7 @@
       </c>
       <c r="G77" s="171" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -17498,7 +17498,7 @@
       </c>
       <c r="G79" s="171" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
     </row>
@@ -23211,9 +23211,9 @@
     <mergeCell ref="C81:F81"/>
     <mergeCell ref="C216:G216"/>
     <mergeCell ref="C186:F186"/>
+    <mergeCell ref="A230:G230"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="C217:F217"/>
-    <mergeCell ref="A230:G230"/>
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="C136:F136"/>
     <mergeCell ref="C210:F210"/>

</xml_diff>